<commit_message>
Add formatted Excel traffic analysis report
</commit_message>
<xml_diff>
--- a/traffic_analysis.xlsx
+++ b/traffic_analysis.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Traffic Analysis" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,302 +413,316 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Time</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Cars</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Bikes</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Buses</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Trucks</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Total</t>
+          <t>Hourly Traffic Volume Analysis</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>07:00</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>120</v>
-      </c>
-      <c r="C2" t="n">
-        <v>85</v>
-      </c>
-      <c r="D2" t="n">
-        <v>12</v>
-      </c>
-      <c r="E2" t="n">
-        <v>18</v>
-      </c>
-      <c r="F2" t="n">
-        <v>235</v>
+          <t>Traffic Data Analysis Using Python</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>08:00</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>245</v>
-      </c>
-      <c r="C3" t="n">
-        <v>160</v>
-      </c>
-      <c r="D3" t="n">
-        <v>20</v>
-      </c>
-      <c r="E3" t="n">
-        <v>25</v>
-      </c>
-      <c r="F3" t="n">
-        <v>450</v>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Cars</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Bikes</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Buses</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Trucks</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>215</v>
+        <v>120</v>
       </c>
       <c r="C4" t="n">
-        <v>150</v>
+        <v>85</v>
       </c>
       <c r="D4" t="n">
+        <v>12</v>
+      </c>
+      <c r="E4" t="n">
         <v>18</v>
       </c>
-      <c r="E4" t="n">
-        <v>22</v>
-      </c>
       <c r="F4" t="n">
-        <v>405</v>
+        <v>235</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>180</v>
+        <v>245</v>
       </c>
       <c r="C5" t="n">
-        <v>130</v>
+        <v>160</v>
       </c>
       <c r="D5" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E5" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F5" t="n">
-        <v>345</v>
+        <v>450</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>170</v>
+        <v>215</v>
       </c>
       <c r="C6" t="n">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="D6" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="E6" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F6" t="n">
-        <v>322</v>
+        <v>405</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>190</v>
+        <v>180</v>
       </c>
       <c r="C7" t="n">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="D7" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E7" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F7" t="n">
-        <v>367</v>
+        <v>345</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>210</v>
+        <v>170</v>
       </c>
       <c r="C8" t="n">
-        <v>155</v>
+        <v>120</v>
       </c>
       <c r="D8" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="F8" t="n">
-        <v>405</v>
+        <v>322</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>220</v>
+        <v>190</v>
       </c>
       <c r="C9" t="n">
-        <v>165</v>
+        <v>140</v>
       </c>
       <c r="D9" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E9" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F9" t="n">
-        <v>428</v>
+        <v>367</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>240</v>
+        <v>210</v>
       </c>
       <c r="C10" t="n">
-        <v>175</v>
+        <v>155</v>
       </c>
       <c r="D10" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E10" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F10" t="n">
-        <v>461</v>
+        <v>405</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>260</v>
+        <v>220</v>
       </c>
       <c r="C11" t="n">
-        <v>190</v>
+        <v>165</v>
       </c>
       <c r="D11" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E11" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="F11" t="n">
-        <v>500</v>
+        <v>428</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>310</v>
+        <v>240</v>
       </c>
       <c r="C12" t="n">
-        <v>230</v>
+        <v>175</v>
       </c>
       <c r="D12" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="E12" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F12" t="n">
-        <v>595</v>
+        <v>461</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>260</v>
+      </c>
+      <c r="C13" t="n">
+        <v>190</v>
+      </c>
+      <c r="D13" t="n">
+        <v>22</v>
+      </c>
+      <c r="E13" t="n">
+        <v>28</v>
+      </c>
+      <c r="F13" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>310</v>
+      </c>
+      <c r="C14" t="n">
+        <v>230</v>
+      </c>
+      <c r="D14" t="n">
+        <v>25</v>
+      </c>
+      <c r="E14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F14" t="n">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>18:00</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="B15" t="n">
         <v>280</v>
       </c>
-      <c r="C13" t="n">
+      <c r="C15" t="n">
         <v>210</v>
       </c>
-      <c r="D13" t="n">
+      <c r="D15" t="n">
         <v>24</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E15" t="n">
         <v>27</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F15" t="n">
         <v>541</v>
       </c>
     </row>

</xml_diff>